<commit_message>
Fix: limpieza de archivos y correcciones de workflow
</commit_message>
<xml_diff>
--- a/docs/Justificación Decisiones - DonaTrack - Grupo 7.xlsx
+++ b/docs/Justificación Decisiones - DonaTrack - Grupo 7.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="262">
   <si>
     <t>Ambito de decision 
 (Objetos / Arquitectura / Persistencia / Otro)</t>
@@ -714,6 +714,144 @@
   </si>
   <si>
     <t>Agiliza drásticamente el ciclo de desarrollo y pruebas. Permite iniciar el sistema y tener instantáneamente objetos válidos para testear los flujos complejos (ej. planificar un camión) sin perder tiempo en configuraciones previas.</t>
+  </si>
+  <si>
+    <t>ENTREGA 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Persistencia / 
+Arquitectura </t>
+  </si>
+  <si>
+    <t>Módulo donatrack-logistica vs. donaciones, incentivos, notificaciones</t>
+  </si>
+  <si>
+    <t>Adopción de Persistencia Políglota: Migración del servicio de Logística a base de datos documental (MongoDB) mediante ODM (Spring Data MongoDB), manteniendo PostgreSQL relacional con JPA/Hibernate para Donaciones, Incentivos y Notificaciones.</t>
+  </si>
+  <si>
+    <t>- Mantener PostgreSQL único para todos los microservicios.
+- Migrar todo el ecosistema DonaTrack a MongoDB.
+- Utilizar base de datos clave-valor (Redis) o grafos (Neo4j) para logística.</t>
+  </si>
+  <si>
+    <t>MongoDB permite lecturas completas en O(1)O(1) sin JOINs. En contraste, Donaciones e Incentivos exigen consistencia ACID estricta, restricciones de integridad referencial y auditoría contable/transaccional que PostgreSQL resuelve de forma óptima.</t>
+  </si>
+  <si>
+    <t>Entidades de Reparto (RutaDeReparto, Parada, Entrega, ComprobanteRecepcion)</t>
+  </si>
+  <si>
+    <t>Patrón Agregado Raíz Documental: Modelar RutaDeRepartoDocument como documento raíz en la colección rutas_reparto, embebiendo la lista de ParadaDocument y dentro de cada parada la lista de EntregaDocument con sus comprobantes.</t>
+  </si>
+  <si>
+    <t>- Normalizar en colecciones separadas (paradas, entregas) vinculadas por ObjectIds o DBRefs.
+- Guardar únicamente la ruta plana y resolver las paradas en memoria.</t>
+  </si>
+  <si>
+    <t>En el modelo de dominio de distribución, las paradas y entregas no tienen sentido ni ciclo de vida fuera de su ruta asignada. Embeberlas garantiza operaciones de lectura y actualización atómicas nativas a nivel de documento en MongoDB, eliminando completamente la necesidad de 5 JOINs o múltiples queries independientes.</t>
+  </si>
+  <si>
+    <t>CamionDocument, ChoferDocument dentro de RutaDeRepartoDocument</t>
+  </si>
+  <si>
+    <t>Desnormalización Estratégica con Snapshot Histórico: Desnormalizar atributos clave del camión (patente, capacidadCarga, capacidadVolumen, altura) y del chofer (legajo, nombre) directamente en el documento de la ruta.</t>
+  </si>
+  <si>
+    <t>- Guardar solo camionId y choferId y consultar maestros mediante $lookup en MongoDB o llamadas REST inter-servicios.</t>
+  </si>
+  <si>
+    <t>1. Lectura O(1)O(1): El chofer consulta su hoja de ruta diaria en una única operación sin cruzar colecciones.
+2. Snapshot Inmutable: Garantiza que si un camión cambia de capacidades o un chofer es desvinculado a futuro, los viajes históricos cerrados preserven exactamente las condiciones y el responsable con que fueron realizados.</t>
+  </si>
+  <si>
+    <t>ComprobanteRecepcion (Fotos y comprobante de entrega)</t>
+  </si>
+  <si>
+    <t>Almacenamiento Semi-Estructurado Nativo: Persistir la lista de URLs de fotos (List&lt;String&gt; fotos) como un array BSON nativo dentro del subdocumento ComprobanteRecepcionDocument.</t>
+  </si>
+  <si>
+    <t>- Crear tabla o colección intermedia comprobante_fotos.
+- Almacenar los binarios directamente en Base64 o GridFS.</t>
+  </si>
+  <si>
+    <t>Las fotografías residen en almacenamiento de objetos en la nube (S3 o similares) y la base almacena solo sus URLs. El soporte nativo de arrays en BSON elimina la impedancia objeto-relacional y no consume espacio innecesario en la base de datos.</t>
+  </si>
+  <si>
+    <t>Límite BSON (16 MB) en RutaDeRepartoDocument</t>
+  </si>
+  <si>
+    <t>Validación de Cota Máxima de Tamaño: Establecer una cota operativa de hasta 100 paradas/entregas por hoja de ruta, verificando que el documento promedio ronde entre 15 KB y 50 KB (menos del 0.3% del límite de 16 MB de MongoDB).</t>
+  </si>
+  <si>
+    <t>- Fragmentar hojas de ruta en múltiples documentos mediante paginación física.
+- Utilizar almacenamiento GridFS para documentos grandes.</t>
+  </si>
+  <si>
+    <t>Con un máximo de 100 entregas por jornada laboral de camión, el documento se mantiene órdenes de magnitud por debajo del tope de BSON, asegurando un consumo mínimo de memoria RAM y máximo rendimiento en cache (WiredTiger).</t>
+  </si>
+  <si>
+    <t>Consulta de Entrega por ID de Donación (/api/entregas/:idDonacion/confirmar)</t>
+  </si>
+  <si>
+    <t>Indexación Compuesta Multinivel: Crear el índice @CompoundIndex(name = "idx_entregas_id", def = "{'paradas.entregas.idEntrega': 1}") en RutaDeRepartoDocument.</t>
+  </si>
+  <si>
+    <t>- Mantener una colección auxiliar de lookup inverso (entregas_lookup).
+- Realizar escaneo completo de colección (ColScan).</t>
+  </si>
+  <si>
+    <t>Permite a los choferes y beneficiarios confirmar entregas o reportar fallas referenciando directamente el UUID de la donación original, permitiendo a MongoDB ubicar la ruta contenedora en tiempo logarítmico O(log⁡N)O(logN) sin full scan.</t>
+  </si>
+  <si>
+    <t>Capa de Infraestructura (donatrack-logistica)</t>
+  </si>
+  <si>
+    <t>Aislamiento Estricto en Arquitectura Hexagonal: Implementar los adaptadores de MongoDB (MongoCamionRepository, MongoRutaDeRepartoRepository, etc.) implementando los Puertos de Salida existentes (CamionRepositoryPort, RutaDeRepartoRepositoryPort), sin modificar el Dominio ni los Casos de Uso.</t>
+  </si>
+  <si>
+    <t>- Anotar directamente las entidades de dominio con @Document de Spring Data.
+- Acoplar los Casos de Uso a interfaces MongoRepository.</t>
+  </si>
+  <si>
+    <t>Cumple con el Principio de Inversión de Dependencias (DIP) y Clean Architecture. El Dominio y la Lógica de Negocio permanecen 100% agnósticos al motor de persistencia, demostrando la verdadera reusabilidad de la arquitectura hexagonal ante cambios de base de datos.</t>
+  </si>
+  <si>
+    <t>Estrategia de Perfiles de Despliegue (local vs. prod)</t>
+  </si>
+  <si>
+    <t>Desacople entre Perfil de Spring y Entorno de Cliente: Configurar perfiles de Spring (local para Docker Mongo/Postgres vs. prod para Atlas/Supabase) y entornos de Bruno (dev para localhost vs. prod para Render en la nube).</t>
+  </si>
+  <si>
+    <t>- Mantener una única configuración apuntando siempre a la nube.
+- Depender de flags de compilación o variables cableadas en código.</t>
+  </si>
+  <si>
+    <t>Confiere flexibilidad total al equipo: se puede desarrollar localmente sin internet mediante Docker Compose, o levantar los servicios apuntando a MongoDB Atlas y Supabase en la nube para pruebas reales, seleccionando dev en Bruno para pegarle al puerto local.</t>
+  </si>
+  <si>
+    <t>Poblado Inicial de Datos (Seeding en MongoDB)</t>
+  </si>
+  <si>
+    <t>Estrategia Dual de Precarga: Creación del script /database/mongo-init.js montado en el contenedor Docker, combinado con un componente Spring Boot MongoDataInitializer (CommandLineRunner) que auto-puebla camiones, choferes, items y rutas si la base está vacía.</t>
+  </si>
+  <si>
+    <t>- Carga manual requerida por el evaluador mediante llamadas HTTP.
+- Scripts de shell externos para ejecutar tras levantar contenedores.</t>
+  </si>
+  <si>
+    <t>Garantiza la paridad de experiencia con PostgreSQL (que ya poseía init.sql y local-seed-data.sql). Tanto en Docker local como en MongoDB Atlas, el sistema arranca con datos de prueba consistentes listos para usar en Bruno y en la defensa.</t>
+  </si>
+  <si>
+    <t>Colección de Bruno para Logística</t>
+  </si>
+  <si>
+    <t>Reescritura, Corrección y Secuenciación Integral: Refactorización completa de los 17 archivos .yml en docs/donatrack-api/Donatrack - API/Logistica/, corrigiendo campos inexistentes, ajustando contratos de dominio (camión y chofer embebidos en callback) e incorporando endpoints CRUD completos (seq: 1..17).</t>
+  </si>
+  <si>
+    <t>- Probar únicamente mediante tests automatizados JUnit sin actualizar Bruno.
+- Mantener llamadas desactualizadas de entregas anteriores.</t>
+  </si>
+  <si>
+    <t>Ofrece una suite de verificación interactiva y reproducible al 100% con respuestas HTTP 200 OK, permitiendo al docente o evaluador inspeccionar en tiempo real cómo impactan los datos en MongoDB local o Atlas.</t>
   </si>
 </sst>
 </file>
@@ -826,7 +964,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -864,6 +1002,9 @@
     </xf>
     <xf borderId="5" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2012,31 +2153,205 @@
       </c>
     </row>
     <row r="57" ht="15.75" customHeight="1">
-      <c r="A57" s="5"/>
-      <c r="B57" s="11"/>
-      <c r="C57" s="11"/>
-      <c r="D57" s="11"/>
-      <c r="E57" s="11"/>
+      <c r="A57" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="B57" s="3"/>
+      <c r="C57" s="3"/>
+      <c r="D57" s="3"/>
+      <c r="E57" s="4"/>
     </row>
     <row r="58" ht="15.75" customHeight="1">
-      <c r="A58" s="5"/>
-      <c r="B58" s="11"/>
-      <c r="C58" s="11"/>
-      <c r="D58" s="11"/>
-      <c r="E58" s="11"/>
-    </row>
-    <row r="59" ht="15.75" customHeight="1"/>
-    <row r="60" ht="15.75" customHeight="1"/>
-    <row r="61" ht="15.75" customHeight="1"/>
-    <row r="62" ht="15.75" customHeight="1"/>
-    <row r="63" ht="15.75" customHeight="1"/>
-    <row r="64" ht="15.75" customHeight="1"/>
-    <row r="65" ht="15.75" customHeight="1"/>
-    <row r="66" ht="15.75" customHeight="1"/>
-    <row r="67" ht="15.75" customHeight="1"/>
-    <row r="68" ht="15.75" customHeight="1"/>
-    <row r="69" ht="15.75" customHeight="1"/>
-    <row r="70" ht="15.75" customHeight="1"/>
+      <c r="A58" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="B58" s="11" t="s">
+        <v>222</v>
+      </c>
+      <c r="C58" s="11" t="s">
+        <v>223</v>
+      </c>
+      <c r="D58" s="11" t="s">
+        <v>224</v>
+      </c>
+      <c r="E58" s="11" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="59" ht="15.75" customHeight="1">
+      <c r="A59" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B59" s="11" t="s">
+        <v>226</v>
+      </c>
+      <c r="C59" s="11" t="s">
+        <v>227</v>
+      </c>
+      <c r="D59" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="E59" s="11" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="60" ht="15.75" customHeight="1">
+      <c r="A60" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B60" s="11" t="s">
+        <v>230</v>
+      </c>
+      <c r="C60" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="D60" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="E60" s="11" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="61" ht="15.75" customHeight="1">
+      <c r="A61" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B61" s="11" t="s">
+        <v>234</v>
+      </c>
+      <c r="C61" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="D61" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="E61" s="11" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="62" ht="15.75" customHeight="1">
+      <c r="A62" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="B62" s="11" t="s">
+        <v>238</v>
+      </c>
+      <c r="C62" s="11" t="s">
+        <v>239</v>
+      </c>
+      <c r="D62" s="11" t="s">
+        <v>240</v>
+      </c>
+      <c r="E62" s="11" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="63" ht="15.75" customHeight="1">
+      <c r="A63" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="B63" s="11" t="s">
+        <v>242</v>
+      </c>
+      <c r="C63" s="11" t="s">
+        <v>243</v>
+      </c>
+      <c r="D63" s="11" t="s">
+        <v>244</v>
+      </c>
+      <c r="E63" s="11" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="64" ht="15.75" customHeight="1">
+      <c r="A64" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B64" s="11" t="s">
+        <v>246</v>
+      </c>
+      <c r="C64" s="11" t="s">
+        <v>247</v>
+      </c>
+      <c r="D64" s="11" t="s">
+        <v>248</v>
+      </c>
+      <c r="E64" s="11" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="65" ht="15.75" customHeight="1">
+      <c r="A65" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B65" s="11" t="s">
+        <v>250</v>
+      </c>
+      <c r="C65" s="11" t="s">
+        <v>251</v>
+      </c>
+      <c r="D65" s="11" t="s">
+        <v>252</v>
+      </c>
+      <c r="E65" s="11" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="66" ht="15.75" customHeight="1">
+      <c r="A66" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="B66" s="11" t="s">
+        <v>254</v>
+      </c>
+      <c r="C66" s="11" t="s">
+        <v>255</v>
+      </c>
+      <c r="D66" s="11" t="s">
+        <v>256</v>
+      </c>
+      <c r="E66" s="11" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="67" ht="15.75" customHeight="1">
+      <c r="A67" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="B67" s="11" t="s">
+        <v>258</v>
+      </c>
+      <c r="C67" s="11" t="s">
+        <v>259</v>
+      </c>
+      <c r="D67" s="11" t="s">
+        <v>260</v>
+      </c>
+      <c r="E67" s="11" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="68" ht="15.75" customHeight="1">
+      <c r="A68" s="14"/>
+      <c r="B68" s="11"/>
+      <c r="C68" s="11"/>
+      <c r="D68" s="11"/>
+      <c r="E68" s="11"/>
+    </row>
+    <row r="69" ht="15.75" customHeight="1">
+      <c r="A69" s="5"/>
+      <c r="B69" s="11"/>
+      <c r="C69" s="11"/>
+      <c r="D69" s="11"/>
+      <c r="E69" s="11"/>
+    </row>
+    <row r="70" ht="15.75" customHeight="1">
+      <c r="A70" s="5"/>
+      <c r="B70" s="11"/>
+      <c r="C70" s="11"/>
+      <c r="D70" s="11"/>
+      <c r="E70" s="11"/>
+    </row>
     <row r="71" ht="15.75" customHeight="1"/>
     <row r="72" ht="15.75" customHeight="1"/>
     <row r="73" ht="15.75" customHeight="1"/>
@@ -2984,12 +3299,25 @@
     <row r="1015" ht="15.75" customHeight="1"/>
     <row r="1016" ht="15.75" customHeight="1"/>
     <row r="1017" ht="15.75" customHeight="1"/>
+    <row r="1018" ht="15.75" customHeight="1"/>
+    <row r="1019" ht="15.75" customHeight="1"/>
+    <row r="1020" ht="15.75" customHeight="1"/>
+    <row r="1021" ht="15.75" customHeight="1"/>
+    <row r="1022" ht="15.75" customHeight="1"/>
+    <row r="1023" ht="15.75" customHeight="1"/>
+    <row r="1024" ht="15.75" customHeight="1"/>
+    <row r="1025" ht="15.75" customHeight="1"/>
+    <row r="1026" ht="15.75" customHeight="1"/>
+    <row r="1027" ht="15.75" customHeight="1"/>
+    <row r="1028" ht="15.75" customHeight="1"/>
+    <row r="1029" ht="15.75" customHeight="1"/>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A18:E18"/>
     <mergeCell ref="A29:E29"/>
     <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A57:E57"/>
   </mergeCells>
   <dataValidations>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C3 C22">

</xml_diff>